<commit_message>
checking final details for resubmission
</commit_message>
<xml_diff>
--- a/data/SSC/turb_threshold/turbidity_threshold_selection.xlsx
+++ b/data/SSC/turb_threshold/turbidity_threshold_selection.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nicol\Documents\sediment_trap_paper\data\SSC\turb_threshold\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08B8386A-5AA7-4220-B44D-D6C93103286C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABD8D7B4-923A-4CCA-805B-DAE78BEF9F23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{54B3BA04-87A9-4FFC-AD84-7319B42309EF}"/>
+    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{54B3BA04-87A9-4FFC-AD84-7319B42309EF}"/>
   </bookViews>
   <sheets>
     <sheet name="SSC-turb" sheetId="5" r:id="rId1"/>
@@ -2217,16 +2217,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B4CAA72-DA07-449E-AC29-192D35BE5032}">
   <dimension ref="A1:R73"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.44140625" customWidth="1"/>
-    <col min="11" max="11" width="20.109375" customWidth="1"/>
-    <col min="13" max="13" width="11.44140625" customWidth="1"/>
-    <col min="14" max="14" width="13.88671875" customWidth="1"/>
-    <col min="15" max="15" width="14.33203125" customWidth="1"/>
+    <col min="1" max="1" width="18.42578125" customWidth="1"/>
+    <col min="11" max="11" width="20.140625" customWidth="1"/>
+    <col min="13" max="13" width="11.42578125" customWidth="1"/>
+    <col min="14" max="14" width="13.85546875" customWidth="1"/>
+    <col min="15" max="15" width="14.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -2258,7 +2258,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>45033.6875</v>
       </c>
@@ -2298,7 +2298,7 @@
       </c>
       <c r="R2" s="14"/>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>45033.854166666664</v>
       </c>
@@ -2344,7 +2344,7 @@
         <v>6.385618</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
         <v>45034.020833333336</v>
       </c>
@@ -2390,7 +2390,7 @@
         <v>38.996000000000002</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
         <v>45034.1875</v>
       </c>
@@ -2436,7 +2436,7 @@
         <v>15.846865774782607</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
         <v>45034.6875</v>
       </c>
@@ -2482,7 +2482,7 @@
         <v>12.6710177</v>
       </c>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
         <v>45034.895833333336</v>
       </c>
@@ -2514,7 +2514,7 @@
         <v>29.957999999999998</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
         <v>45035.104166666664</v>
       </c>
@@ -2546,7 +2546,7 @@
         <v>22.63</v>
       </c>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A9" s="3">
         <v>45035.3125</v>
       </c>
@@ -2586,7 +2586,7 @@
       </c>
       <c r="R9" s="14"/>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A10" s="3">
         <v>45035.9375</v>
       </c>
@@ -2632,7 +2632,7 @@
         <v>2.4089349000000002</v>
       </c>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A11" s="3">
         <v>45036.145833333336</v>
       </c>
@@ -2678,7 +2678,7 @@
         <v>9.0860785666666608</v>
       </c>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A12" s="3">
         <v>45036.979166666664</v>
       </c>
@@ -2724,7 +2724,7 @@
         <v>5.3451238555555536</v>
       </c>
     </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A13" s="3">
         <v>45037.8125</v>
       </c>
@@ -2770,7 +2770,7 @@
         <v>4.5403580999999997</v>
       </c>
     </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A14" s="3">
         <v>45038.229166666664</v>
       </c>
@@ -2804,7 +2804,7 @@
       </c>
       <c r="R14" s="12"/>
     </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A15" s="3">
         <v>45038.645833333336</v>
       </c>
@@ -2836,7 +2836,7 @@
         <v>22.608116800000001</v>
       </c>
     </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A16" s="3">
         <v>45038.854166666664</v>
       </c>
@@ -2868,7 +2868,7 @@
         <v>15.424431200000001</v>
       </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" s="3">
         <v>45040.083333333336</v>
       </c>
@@ -2900,7 +2900,7 @@
         <v>13.66403352</v>
       </c>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A18" s="3">
         <v>45040.708333333336</v>
       </c>
@@ -2932,7 +2932,7 @@
         <v>11.230658699999999</v>
       </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" s="3">
         <v>45040.916666666664</v>
       </c>
@@ -2964,7 +2964,7 @@
         <v>8.7104481200000006</v>
       </c>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" s="3">
         <v>45044.666666666664</v>
       </c>
@@ -2996,7 +2996,7 @@
         <v>22.608116800000001</v>
       </c>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" s="3">
         <v>45046.541666666664</v>
       </c>
@@ -3028,7 +3028,7 @@
         <v>14.398190400000001</v>
       </c>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" s="3">
         <v>45046.75</v>
       </c>
@@ -3060,7 +3060,7 @@
         <v>11.250394099999999</v>
       </c>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A23" s="3">
         <v>45047.833333333336</v>
       </c>
@@ -3092,7 +3092,7 @@
         <v>9.6024881999999998</v>
       </c>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A24" s="3">
         <v>45049.583333333336</v>
       </c>
@@ -3124,7 +3124,7 @@
         <v>8.7834690999999996</v>
       </c>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" s="3">
         <v>45049.833333333336</v>
       </c>
@@ -3156,7 +3156,7 @@
         <v>7.0862246999999998</v>
       </c>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A26" s="3"/>
       <c r="B26" s="2"/>
       <c r="C26" s="1"/>
@@ -3178,7 +3178,7 @@
         <v>6.9382092000000002</v>
       </c>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27" s="3"/>
       <c r="B27" s="2"/>
       <c r="C27" s="1"/>
@@ -3200,7 +3200,7 @@
         <v>6.385618</v>
       </c>
     </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28" s="3"/>
       <c r="B28" s="2"/>
       <c r="C28" s="1"/>
@@ -3222,7 +3222,7 @@
         <v>7.1355632</v>
       </c>
     </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A29" s="3"/>
       <c r="B29" s="2"/>
       <c r="C29" s="1"/>
@@ -3244,7 +3244,7 @@
         <v>8.6749244000000001</v>
       </c>
     </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:15" x14ac:dyDescent="0.25">
       <c r="K30" s="3">
         <v>45151.885416666664</v>
       </c>
@@ -3261,7 +3261,7 @@
         <v>8.9413523000000001</v>
       </c>
     </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A31" s="3">
         <v>45034.354166666664</v>
       </c>
@@ -3293,7 +3293,7 @@
         <v>7.8953761</v>
       </c>
     </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A32" s="3">
         <v>45034.520833333336</v>
       </c>
@@ -3325,7 +3325,7 @@
         <v>13.497999999999999</v>
       </c>
     </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A33" s="3">
         <v>45035.520833333336</v>
       </c>
@@ -3357,7 +3357,7 @@
         <v>13.875999999999999</v>
       </c>
     </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A34" s="3">
         <v>45035.729166666664</v>
       </c>
@@ -3389,7 +3389,7 @@
         <v>12.423999999999999</v>
       </c>
     </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A35" s="3">
         <v>45036.354166666664</v>
       </c>
@@ -3421,7 +3421,7 @@
         <v>9.9559999999999995</v>
       </c>
     </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A36" s="3">
         <v>45036.770833333336</v>
       </c>
@@ -3453,7 +3453,7 @@
         <v>35.663083899999997</v>
       </c>
     </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A37" s="3">
         <v>45037.395833333336</v>
       </c>
@@ -3469,6 +3469,10 @@
       <c r="E37" s="1">
         <v>7.9286783333333304</v>
       </c>
+      <c r="G37">
+        <f>73-31</f>
+        <v>42</v>
+      </c>
       <c r="K37" s="3">
         <v>45166.524305555555</v>
       </c>
@@ -3485,7 +3489,7 @@
         <v>24.996100200000001</v>
       </c>
     </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A38" s="3">
         <v>45037.604166666664</v>
       </c>
@@ -3517,7 +3521,7 @@
         <v>15.3060188</v>
       </c>
     </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A39" s="3">
         <v>45038.020833333336</v>
       </c>
@@ -3549,7 +3553,7 @@
         <v>12.918035400000001</v>
       </c>
     </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A40" s="3">
         <v>45038.4375</v>
       </c>
@@ -3581,7 +3585,7 @@
         <v>11.4082773</v>
       </c>
     </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A41" s="3">
         <v>45039.0625</v>
       </c>
@@ -3613,7 +3617,7 @@
         <v>10.678067499999999</v>
       </c>
     </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A42" s="3">
         <v>45039.666666666664</v>
       </c>
@@ -3645,7 +3649,7 @@
         <v>10.9346277</v>
       </c>
     </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A43" s="3">
         <v>45039.875</v>
       </c>
@@ -3677,7 +3681,7 @@
         <v>12.23</v>
       </c>
     </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A44" s="3">
         <v>45040.291666666664</v>
       </c>
@@ -3709,7 +3713,7 @@
         <v>14.09</v>
       </c>
     </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A45" s="3">
         <v>45041.125</v>
       </c>
@@ -3741,7 +3745,7 @@
         <v>13.07</v>
       </c>
     </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A46" s="3">
         <v>45041.541666666664</v>
       </c>
@@ -3773,7 +3777,7 @@
         <v>10.54</v>
       </c>
     </row>
-    <row r="47" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A47" s="3">
         <v>45041.75</v>
       </c>
@@ -3803,7 +3807,7 @@
         <v>8.4700000000000006</v>
       </c>
     </row>
-    <row r="48" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A48" s="3">
         <v>45042.5625</v>
       </c>
@@ -3820,7 +3824,7 @@
         <v>6.9584305310000003</v>
       </c>
     </row>
-    <row r="49" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A49" s="3">
         <v>45042.791666666664</v>
       </c>
@@ -3852,7 +3856,7 @@
         <v>4.5403580999999997</v>
       </c>
     </row>
-    <row r="50" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A50" s="3">
         <v>45043</v>
       </c>
@@ -3884,7 +3888,7 @@
         <v>2.4089349000000002</v>
       </c>
     </row>
-    <row r="51" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A51" s="3">
         <v>45043.208333333336</v>
       </c>
@@ -3916,7 +3920,7 @@
         <v>9.0860785666666608</v>
       </c>
     </row>
-    <row r="52" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A52" s="3">
         <v>45043.625</v>
       </c>
@@ -3933,7 +3937,7 @@
         <v>8.7752321066666603</v>
       </c>
     </row>
-    <row r="53" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A53" s="3">
         <v>45044.041666666664</v>
       </c>
@@ -3950,7 +3954,7 @@
         <v>8.3964748666666598</v>
       </c>
     </row>
-    <row r="54" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A54" s="3">
         <v>45044.25</v>
       </c>
@@ -3967,7 +3971,7 @@
         <v>11.483500266666599</v>
       </c>
     </row>
-    <row r="55" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A55" s="3">
         <v>45044.458333333336</v>
       </c>
@@ -3984,7 +3988,7 @@
         <v>5.4046995333333303</v>
       </c>
     </row>
-    <row r="56" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A56" s="3">
         <v>45044.875</v>
       </c>
@@ -4001,7 +4005,7 @@
         <v>5.62346873333333</v>
       </c>
     </row>
-    <row r="57" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A57" s="3">
         <v>45045.083333333336</v>
       </c>
@@ -4018,7 +4022,7 @@
         <v>6.59702113333333</v>
       </c>
     </row>
-    <row r="58" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A58" s="3">
         <v>45045.5</v>
       </c>
@@ -4035,7 +4039,7 @@
         <v>4.8982727333333296</v>
       </c>
     </row>
-    <row r="59" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A59" s="3">
         <v>45045.708333333336</v>
       </c>
@@ -4052,7 +4056,7 @@
         <v>12.434267999999999</v>
       </c>
     </row>
-    <row r="60" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A60" s="3">
         <v>45045.916666666664</v>
       </c>
@@ -4069,7 +4073,7 @@
         <v>8.70769666666666</v>
       </c>
     </row>
-    <row r="61" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A61" s="3">
         <v>45046.125</v>
       </c>
@@ -4086,7 +4090,7 @@
         <v>10.258584000000001</v>
       </c>
     </row>
-    <row r="62" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A62" s="3">
         <v>45046.333333333336</v>
       </c>
@@ -4103,7 +4107,7 @@
         <v>7.5019323999999896</v>
       </c>
     </row>
-    <row r="63" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A63" s="3">
         <v>45046.958333333336</v>
       </c>
@@ -4120,7 +4124,7 @@
         <v>20.852958666666598</v>
       </c>
     </row>
-    <row r="64" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A64" s="3">
         <v>45047.166666666664</v>
       </c>
@@ -4137,7 +4141,7 @@
         <v>12.526063343999899</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" s="3">
         <v>45047.375</v>
       </c>
@@ -4154,7 +4158,7 @@
         <v>9.3400750666666603</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" s="3">
         <v>45047.583333333336</v>
       </c>
@@ -4171,7 +4175,7 @@
         <v>12.602335333333301</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" s="3">
         <v>45048.125</v>
       </c>
@@ -4188,7 +4192,7 @@
         <v>12.6200733333333</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" s="3">
         <v>45048.708333333336</v>
       </c>
@@ -4205,7 +4209,7 @@
         <v>10.38581286</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" s="3">
         <v>45049</v>
       </c>
@@ -4222,7 +4226,7 @@
         <v>8.9650455999999998</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" s="3">
         <v>45049.291666666664</v>
       </c>
@@ -4239,7 +4243,7 @@
         <v>9.1913850666666601</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" s="3">
         <v>45050.208333333336</v>
       </c>
@@ -4256,7 +4260,7 @@
         <v>11.1430651333333</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" s="3">
         <v>45050.583333333336</v>
       </c>
@@ -4273,7 +4277,7 @@
         <v>10.366192399999999</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" s="3">
         <v>45051.208333333336</v>
       </c>

</xml_diff>